<commit_message>
fix(pipeline): sanitiza caracteres ilegais no excel e atualiza base parquet
</commit_message>
<xml_diff>
--- a/outputs/senai_relatorio_qualidade.xlsx
+++ b/outputs/senai_relatorio_qualidade.xlsx
@@ -15,6 +15,9 @@
     <sheet name="04_Rateio de Despesas (SENA" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="05_Despesas por Licitação (" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="06_Bens Imóveis (SENAI - SE" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="07_Relação de Dirigentes e" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="08_Composição do Conselho (" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="09_Comissão de Contas e Orç" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -501,7 +504,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Execução Orçamentária (SENAI - SENAI-DN - 2025)</t>
+          <t>Execução Orçamentária (SENAI - SENAI-DN - 2024)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -511,7 +514,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://sorsdn.sistemaindustria.com.br/api/Transparencia/Get?entidade=SENAI&amp;regional=SENAI-DN&amp;ano=2025</t>
+          <t>https://sorsdn.sistemaindustria.com.br/api/Transparencia/Get?entidade=SENAI&amp;regional=SENAI-DN&amp;ano=2024</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -537,7 +540,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-08-13 17:09:49</t>
+          <t>2026-08-17 14:51:22</t>
         </is>
       </c>
     </row>
@@ -557,7 +560,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Saldo Exercício Anterior (SENAI - SENAI-DN - 2025)</t>
+          <t>Saldo Exercício Anterior (SENAI - SENAI-DN - 2024)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -567,7 +570,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://sorsdn.sistemaindustria.com.br/api/Transparencia/GetSaldoExercicioAnterior?entidade=SENAI&amp;regional=SENAI-DN&amp;ano=2025</t>
+          <t>https://sorsdn.sistemaindustria.com.br/api/Transparencia/GetSaldoExercicioAnterior?entidade=SENAI&amp;regional=SENAI-DN&amp;ano=2024</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -593,7 +596,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-08-13 17:09:49</t>
+          <t>2026-08-17 14:51:22</t>
         </is>
       </c>
     </row>
@@ -613,7 +616,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Previsão Orçamentária (SENAI - 2025)</t>
+          <t>Previsão Orçamentária (SENAI - 2024)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -623,7 +626,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://sorsdn.sistemaindustria.com.br/api/Transparencia/GetPrevisaoOrcamentaria?entidade=SENAI&amp;ano=2025</t>
+          <t>https://sorsdn.sistemaindustria.com.br/api/Transparencia/GetPrevisaoOrcamentaria?entidade=SENAI&amp;ano=2024</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -649,7 +652,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-08-13 17:09:49</t>
+          <t>2026-08-17 14:51:22</t>
         </is>
       </c>
     </row>
@@ -669,7 +672,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Rateio de Despesas (SENAI - SENAI-DN - 2025)</t>
+          <t>Rateio de Despesas (SENAI - SENAI-DN - 2024)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -679,7 +682,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://sorsdn.sistemaindustria.com.br/api/Transparencia/GetRateio?entidade=SENAI&amp;regional=SENAI-DN&amp;ano=2025</t>
+          <t>https://sorsdn.sistemaindustria.com.br/api/Transparencia/GetRateio?entidade=SENAI&amp;regional=SENAI-DN&amp;ano=2024</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -705,7 +708,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-08-13 17:09:49</t>
+          <t>2026-08-17 14:51:22</t>
         </is>
       </c>
     </row>
@@ -725,7 +728,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Despesas por Licitação (SENAI - SENAI-DN - 2025)</t>
+          <t>Despesas por Licitação (SENAI - SENAI-DN - 2024)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -735,7 +738,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://sorsdn.sistemaindustria.com.br/api/Transparencia/GetLicitacao?entidade=SENAI&amp;regional=SENAI-DN&amp;ano=2025</t>
+          <t>https://sorsdn.sistemaindustria.com.br/api/Transparencia/GetLicitacao?entidade=SENAI&amp;regional=SENAI-DN&amp;ano=2024</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -761,7 +764,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-08-13 17:09:49</t>
+          <t>2026-08-17 14:51:22</t>
         </is>
       </c>
     </row>
@@ -781,7 +784,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Bens Imóveis (SENAI - SENAI-DN - 2025)</t>
+          <t>Bens Imóveis (SENAI - SENAI-DN - 2024)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -791,7 +794,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://sorsdn.sistemaindustria.com.br/api/Transparencia/GetBensImoveis?entidade=SENAI&amp;regional=SENAI-DN&amp;ano=2025</t>
+          <t>https://sorsdn.sistemaindustria.com.br/api/Transparencia/GetBensImoveis?entidade=SENAI&amp;regional=SENAI-DN&amp;ano=2024</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -817,7 +820,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-08-13 17:09:49</t>
+          <t>2026-08-17 14:51:22</t>
         </is>
       </c>
     </row>
@@ -837,7 +840,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Relação de Dirigentes e Gestão (SENAI - SENAI-DN - 2025)</t>
+          <t>Relação de Dirigentes e Gestão (SENAI - SENAI-DN - 2024)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -847,31 +850,33 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://sistematransparenciaweb.com.br/api-relacaodirigentes-gestao/publico/relacao-dirigente-empregado/entidades/SENAI/departamentos/SENAI-DN/relacao-dirigente-empregado?ano=2025</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>ERRO</t>
-        </is>
+          <t>https://sistematransparenciaweb.com.br/api-relacaodirigentes-gestao/publico/relacao-dirigente-empregado/entidades/SENAI/departamentos/SENAI-DN/relacao-dirigente-empregado?ano=2024</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>200</v>
       </c>
       <c r="H8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Link inativo (HTTP ERRO)</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr"/>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-08-13 17:09:49</t>
+          <t>2026-08-17 14:51:22</t>
         </is>
       </c>
     </row>
@@ -891,7 +896,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Composição do Conselho (SENAI - SENAI-DN - 2025)</t>
+          <t>Composição do Conselho (SENAI - SENAI-DN - 2024)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -901,31 +906,33 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://sistematransparenciaweb.com.br/api-composicao-conselho/publico/composicao-conselho/entidades/SENAI/departamentos/SENAI-DN/composicao-conselho?ano=2025</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>ERRO</t>
-        </is>
+          <t>https://sistematransparenciaweb.com.br/api-composicao-conselho/publico/composicao-conselho/entidades/SENAI/departamentos/SENAI-DN/composicao-conselho?ano=2024</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>200</v>
       </c>
       <c r="H9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Link inativo (HTTP ERRO)</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr"/>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-08-13 17:09:49</t>
+          <t>2026-08-17 14:51:22</t>
         </is>
       </c>
     </row>
@@ -945,7 +952,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Comissão de Contas e Orçamentos (SENAI - SENAI-DN - 2025)</t>
+          <t>Comissão de Contas e Orçamentos (SENAI - SENAI-DN - 2024)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -955,31 +962,1832 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://sistematransparenciaweb.com.br/api-comissao-contaorcamento/api-comissao-contaorcamento?ano=2025&amp;entidade=SENAI&amp;departamento=SENAI-DN</t>
+          <t>https://sistematransparenciaweb.com.br/api-comissao-contaorcamento/api-comissao-contaorcamento?ano=2024&amp;entidade=SENAI&amp;departamento=SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>200</v>
+      </c>
+      <c r="H10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-08-17 14:51:22</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>codigoComposicaoConselho</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>funcao</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>origem</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>siglaEntidade</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>siglaDepartamento</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>dataPublicacao</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>titulo</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>nota</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>fonte</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>analise</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>extra</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>departamento.nomeDepartamento</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>departamento.siglaEntidadeRegional</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>departamento.uf</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>departamento.cdEntidadeRegionalERP</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>9098</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ALEX DIAS CARVALHO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Conselheiro</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>PRESIDENTE DO CONSELHO REGIONAL - PA</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>9099</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ANTONIO CARLOS DA SILVA </t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Conselheiro</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PRESIDENTE DO CONSELHO REGIONAL - AM</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>9100</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ANTONIO JOSÉ DE MORAES SOUZA FILHO</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Conselheiro</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PRESIDENTE DO CONSELHO REGIONAL - PI</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>9101</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ANTONIO RICARDO ALVAREZ ALBAN</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Presidente do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PRESIDENTE DO CONSELHO NACIONAL </t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>9102</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BRUNO SALVADOR VELOSO DA SILVEIRA</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Conselheiro</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PRESIDENTE DO CONSELHO REGIONAL - PE </t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>9103</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CARLOS HENRIQUE DE OLIVEIRA PASSOS</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Conselheiro</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>PRESIDENTE DO CONSELHO REGIONAL - BA</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>9140</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SÉRGIO MARCOLINO LONGEN </t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Conselheiro</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>PRESIDENTE DO CONSELHO REGIONAL - MS</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>9141</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SILVIO CEZAR PEREIRA RANGEL</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Conselheiro</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>PRESIDENTE DO CONSELHO REGIONAL - MT</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9134</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PAULO CHITOLINA</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Conselheiro</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>CENTRAL ÚNICA DOS TRABALHADORES</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>ERRO</t>
-        </is>
-      </c>
-      <c r="H10" t="b">
-        <v>0</v>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>2024</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>Composição do Conselho Nacional</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Link inativo (HTTP ERRO)</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>2026-08-13 17:09:49</t>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9135</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PEDRO PEREIRA DE SOUSA</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Conselheiro</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>UNIÃO GERAL DOS TRABALHADORES</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>9136</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REPRESENTANTE DO MINISTÉRIO DO TRABALHO E EMPREGO SUPLENTE - AGUARDANDO DESIGNAÇÃO </t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Suplente</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MINISTÉRIO DO TRABALHO E EMPREGO</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>9137</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ROBERTO MAGNO MARTINS PIRES </t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Conselheiro</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>PRESIDENTE DO CONSELHO REGIONAL - TO</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>9138</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ROBERTO PINTO SERQUIZ ELIAS</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Conselheiro</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>PRESIDENTE DO CONSELHO REGIONAL - RN</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>9139</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SANDRO DA MABEL ANTÔNIO SCODRO</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Conselheiro</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>PRESIDENTE DO CONSELHO REGIONAL - GO</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>9128</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>MIGUEL EDUARDO TORRES</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Suplente</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>FORÇA SINDICAL</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>9129</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NELSON LUIZ BONARDI </t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Conselheiro</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>NOVA CENTRAL SINDICAL DE TRABALHADORES</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>9130</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>OSVALDO OLAVIO MAFRA</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Conselheiro</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>FORÇA SINDICAL</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>9131</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PAULA PROENÇA</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Suplente</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>CENTRAL ÚNICA DOS TRABALHADORES</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>9132</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PAULO ALEXANDRE GALLIS PEREIRA BARAONA</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Conselheiro</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>PRESIDENTE DO CONSELHO REGIONAL - ES</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>9133</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>PAULO CEZAR ROSSI</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Suplente</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>UNIÃO GERAL DOS TRABALHADORES</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Composição do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Conselho Nacional do SENAI</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Serviço Nacional de Aprendizagem Industrial</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>03DN0000</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>funcao</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>origem</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>titulo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>nota</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>fonte</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>analise</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>extra</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>dataPublicacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ANTONIO CARLOS DA SILVA </t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MEMBRO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PRESIDENTE DO CONSELHO REGIONAL DO AMAZONAS</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Comissão de Contas</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>A Comissão de Contas foi designada por ato do Conselho Nacional, nos termos do artigo 22 do Regimento do SENAI, para este exercício, com a incumbência de fiscalizar a execução orçamentária, bem como a movimentação de fundos do Departamento Nacional. Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>SENAI/DN</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BRUNO SALVADOR VELOSO DA SILVEIRA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MEMBRO</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PRESIDENTE DO CONSELHO REGIONAL DE PERNAMBUCO</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Comissão de Contas</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>A Comissão de Contas foi designada por ato do Conselho Nacional, nos termos do artigo 22 do Regimento do SENAI, para este exercício, com a incumbência de fiscalizar a execução orçamentária, bem como a movimentação de fundos do Departamento Nacional. Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>SENAI/DN</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CLAUDIO AFONSO AMORETTI BIER</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MEMBRO</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PRESIDENTE DO CONSELHO REGIONAL DO RIO GRANDE DO SUL</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Comissão de Contas</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>A Comissão de Contas foi designada por ato do Conselho Nacional, nos termos do artigo 22 do Regimento do SENAI, para este exercício, com a incumbência de fiscalizar a execução orçamentária, bem como a movimentação de fundos do Departamento Nacional. Não recebem remuneração.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SENAI/DN</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
         </is>
       </c>
     </row>
@@ -1095,7 +2903,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1115,7 +2923,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1133,22 +2941,22 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>1417212825.81</v>
+        <v>1269144085.46</v>
       </c>
       <c r="K2" t="n">
-        <v>1423757320.44</v>
+        <v>1309516069.87</v>
       </c>
       <c r="L2" t="n">
-        <v>100.5</v>
+        <v>103.2</v>
       </c>
       <c r="M2" t="n">
-        <v>75.3</v>
+        <v>80.2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1168,7 +2976,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1190,22 +2998,22 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>368511302.87</v>
+        <v>330012704.85</v>
       </c>
       <c r="K3" t="n">
-        <v>368594797.78</v>
+        <v>338318855.7</v>
       </c>
       <c r="L3" t="n">
-        <v>100</v>
+        <v>102.5</v>
       </c>
       <c r="M3" t="n">
-        <v>19.6</v>
+        <v>20.9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1225,7 +3033,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1247,22 +3055,22 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>430347342.72</v>
+        <v>375353814.35</v>
       </c>
       <c r="K4" t="n">
-        <v>425286354.29</v>
+        <v>391738115.1</v>
       </c>
       <c r="L4" t="n">
-        <v>98.8</v>
+        <v>104.4</v>
       </c>
       <c r="M4" t="n">
-        <v>22.9</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1282,7 +3090,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1304,22 +3112,22 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>618354180.22</v>
+        <v>563777566.26</v>
       </c>
       <c r="K5" t="n">
-        <v>629876168.37</v>
+        <v>579459099.0700001</v>
       </c>
       <c r="L5" t="n">
-        <v>101.9</v>
+        <v>102.8</v>
       </c>
       <c r="M5" t="n">
-        <v>32.9</v>
+        <v>35.6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1339,7 +3147,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1376,7 +3184,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1396,7 +3204,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1433,7 +3241,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1453,7 +3261,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1490,7 +3298,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1510,7 +3318,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1547,7 +3355,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1567,7 +3375,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1604,7 +3412,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1624,7 +3432,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1642,22 +3450,22 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>157144347.16</v>
+        <v>86723319.09999999</v>
       </c>
       <c r="K11" t="n">
-        <v>186719152.4</v>
+        <v>98472941.04000001</v>
       </c>
       <c r="L11" t="n">
-        <v>118.8</v>
+        <v>113.5</v>
       </c>
       <c r="M11" t="n">
-        <v>8.4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1677,7 +3485,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1699,13 +3507,13 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>667374</v>
+        <v>74413.8</v>
       </c>
       <c r="K12" t="n">
-        <v>858593.87</v>
+        <v>132000</v>
       </c>
       <c r="L12" t="n">
-        <v>128.7</v>
+        <v>177.4</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
@@ -1714,7 +3522,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1734,7 +3542,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1756,22 +3564,22 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>156476973.16</v>
+        <v>86648905.3</v>
       </c>
       <c r="K13" t="n">
-        <v>185860558.53</v>
+        <v>98340941.04000001</v>
       </c>
       <c r="L13" t="n">
-        <v>118.8</v>
+        <v>113.5</v>
       </c>
       <c r="M13" t="n">
-        <v>8.300000000000001</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1791,7 +3599,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1824,7 +3632,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1844,7 +3652,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1881,7 +3689,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1901,7 +3709,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1938,7 +3746,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1958,7 +3766,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1976,22 +3784,22 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>150495805.44</v>
+        <v>109726872.65</v>
       </c>
       <c r="K17" t="n">
-        <v>155745946.46</v>
+        <v>120359270.06</v>
       </c>
       <c r="L17" t="n">
-        <v>103.5</v>
+        <v>109.7</v>
       </c>
       <c r="M17" t="n">
-        <v>8</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2011,7 +3819,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2033,22 +3841,22 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>1706423.3</v>
+        <v>10534340.41</v>
       </c>
       <c r="K18" t="n">
-        <v>72726.73</v>
+        <v>60660.32</v>
       </c>
       <c r="L18" t="n">
-        <v>4.3</v>
+        <v>0.6</v>
       </c>
       <c r="M18" t="n">
-        <v>0.1</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2068,7 +3876,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2090,7 +3898,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>1501000</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -2099,13 +3907,13 @@
         <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2125,7 +3933,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2147,22 +3955,22 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>126475000</v>
+        <v>81135400</v>
       </c>
       <c r="K20" t="n">
-        <v>144498863.13</v>
+        <v>101819890</v>
       </c>
       <c r="L20" t="n">
-        <v>114.3</v>
+        <v>125.5</v>
       </c>
       <c r="M20" t="n">
-        <v>6.7</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2182,7 +3990,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2204,7 +4012,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>78103.56</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -2300,7 +4108,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2353,7 +4161,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2406,7 +4214,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2459,7 +4267,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2512,7 +4320,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2565,7 +4373,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2618,7 +4426,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2671,7 +4479,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2804,7 +4612,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>5952293043.34</v>
+        <v>5264101019.49</v>
       </c>
     </row>
     <row r="3">
@@ -2840,7 +4648,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>2463940023.2</v>
+        <v>2200582444.23</v>
       </c>
     </row>
     <row r="4">
@@ -2876,7 +4684,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>2869998839.92</v>
+        <v>2499741009</v>
       </c>
     </row>
     <row r="5">
@@ -2912,7 +4720,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>618354180.22</v>
+        <v>563777566.26</v>
       </c>
     </row>
     <row r="6">
@@ -2944,7 +4752,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>47307000</v>
+        <v>80000000</v>
       </c>
     </row>
     <row r="7">
@@ -2976,7 +4784,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>46368099.6</v>
+        <v>40511947.88</v>
       </c>
     </row>
     <row r="8">
@@ -3008,7 +4816,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>843166709.99</v>
+        <v>488203521.63</v>
       </c>
     </row>
     <row r="9">
@@ -3025,13 +4833,13 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>41010401</t>
+          <t>41010302</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Serviços e Vendas Comerciais</t>
+          <t>Receitas de Artigos Confeccionados em Cursos</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -3040,7 +4848,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>35584189.21</v>
+        <v>750</v>
       </c>
     </row>
     <row r="10">
@@ -3057,13 +4865,13 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>41010402</t>
+          <t>41010401</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Serviços Tecnológicos</t>
+          <t>Serviços e Vendas Comerciais</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -3072,7 +4880,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>558866357.62</v>
+        <v>13427577.52</v>
       </c>
     </row>
     <row r="11">
@@ -3089,13 +4897,13 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>41010403</t>
+          <t>41010402</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Serviços de Consultoria e Assistência Técnica</t>
+          <t>Serviços Tecnológicos</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -3104,7 +4912,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>320933742.55</v>
+        <v>412850667.11</v>
       </c>
     </row>
     <row r="12">
@@ -3121,13 +4929,13 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>41010405</t>
+          <t>41010403</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Serviços Administrativos</t>
+          <t>Serviços de Consultoria e Assistência Técnica</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -3136,7 +4944,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>5949010.35</v>
+        <v>240859837.16</v>
       </c>
     </row>
     <row r="13">
@@ -3153,13 +4961,13 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>41010407</t>
+          <t>41010404</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Serviços de Educacionais</t>
+          <t>Serviços Financeiros</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -3168,7 +4976,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>1498479274.77</v>
+        <v>78608.55</v>
       </c>
     </row>
     <row r="14">
@@ -3185,13 +4993,13 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>41010409</t>
+          <t>41010405</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Serviços Laboratoriais</t>
+          <t>Serviços Administrativos</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -3200,7 +5008,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>82198705.23</v>
+        <v>6622150.08</v>
       </c>
     </row>
     <row r="15">
@@ -3217,13 +5025,13 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>41010501</t>
+          <t>41010407</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Recuperação  de Despesas</t>
+          <t>Serviços de Educacionais</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -3232,7 +5040,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>138967820.68</v>
+        <v>1348206381.25</v>
       </c>
     </row>
     <row r="16">
@@ -3249,13 +5057,13 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>41010502</t>
+          <t>41010409</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Multas e Juros de Mora</t>
+          <t>Serviços Laboratoriais</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -3264,7 +5072,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>12098288.45</v>
+        <v>75692391.84999999</v>
       </c>
     </row>
     <row r="17">
@@ -3281,13 +5089,13 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>41010503</t>
+          <t>41010501</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Descontos Obtidos</t>
+          <t>Recuperação  de Despesas</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -3296,7 +5104,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>1119443.03</v>
+        <v>148818316.05</v>
       </c>
     </row>
     <row r="18">
@@ -3313,13 +5121,13 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>41010504</t>
+          <t>41010502</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>IDENIZACOES, RESTITUICOES E DOACOES</t>
+          <t>Multas e Juros de Mora</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -3328,7 +5136,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>23587620.22</v>
+        <v>77983600.98</v>
       </c>
     </row>
     <row r="19">
@@ -3345,13 +5153,13 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>41010505</t>
+          <t>41010503</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Saldo de Exercícios Anteriores</t>
+          <t>Descontos Obtidos</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -3360,7 +5168,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>7326428</v>
+        <v>2675439.4</v>
       </c>
     </row>
     <row r="20">
@@ -3377,13 +5185,13 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>41010506</t>
+          <t>41010504</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Receitas de Patrocínios</t>
+          <t>IDENIZACOES, RESTITUICOES E DOACOES</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -3392,7 +5200,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>2596575.68</v>
+        <v>48345799.27</v>
       </c>
     </row>
     <row r="21">
@@ -3409,13 +5217,13 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>41020101</t>
+          <t>41010505</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Auxílio Mínimo/Subvenções Ordinárias</t>
+          <t>Saldo de Exercícios Anteriores</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -3424,7 +5232,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>213107441.05</v>
+        <v>13177598</v>
       </c>
     </row>
   </sheetData>
@@ -3497,7 +5305,7 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3507,7 +5315,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Gestão e Suporte às atividades da Diretoria Corporativa</t>
+          <t>Ações de Educação Treinamento e Desenvolvimento</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -3533,7 +5341,7 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3543,25 +5351,25 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Educação Treinamento e Desenvolvimento</t>
+          <t>Gestão de Pessoal e Encargos - Diretoria Corporativa</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Número de Unidades Operacionais e Postos de Atendimentos que prestam atendimento nos Departamentos Regionais do SESI e SENAI e Sede das Federações e do IEL</t>
+          <t>Estabelecido em documento próprio (Ordem de Serviço Remuneração e Encargos CNI/SESI/SENAI/IEL)</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>54.63</v>
+        <v>33</v>
       </c>
       <c r="G3" t="n">
-        <v>42.08</v>
+        <v>33</v>
       </c>
       <c r="H3" t="n">
-        <v>1.71</v>
+        <v>33</v>
       </c>
       <c r="I3" t="n">
-        <v>1.58</v>
+        <v>1</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
@@ -3569,7 +5377,7 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3579,25 +5387,25 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Gestão de Pessoal e Encargos - Diretoria Corporativa</t>
+          <t>Gestão e Suporte às atividades da Diretoria Corporativa</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Estabelecido em documento próprio (Ordem de Serviço Remuneração e Encargos CNI/SESI/SENAI/IEL)</t>
+          <t>Número de Unidades Operacionais e Postos de Atendimentos que prestam atendimento nos Departamentos Regionais do SESI e SENAI e Sede das Federações e do IEL</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>33</v>
+        <v>54.63</v>
       </c>
       <c r="G4" t="n">
-        <v>33</v>
+        <v>42.08</v>
       </c>
       <c r="H4" t="n">
-        <v>33</v>
+        <v>1.71</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>1.58</v>
       </c>
       <c r="J4" t="inlineStr"/>
     </row>
@@ -3605,7 +5413,7 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3615,7 +5423,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Gestão e Suporte as Atividades - Diretoria de Comunicação</t>
+          <t>Ações de Educação Treinamento e Desenvolvimento</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -3641,7 +5449,7 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3651,25 +5459,25 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Gestão de Pessoal e Encargos - Diretoria de Comunicação</t>
+          <t xml:space="preserve">Comunicação - Diretoria de Educação e Tecnologia </t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Número de Unidades Operacionais e Postos de Atendimentos que prestam atendimento nos Departamentos Regionais do SESI e SENAI e Sede das Federações e do IEL</t>
+          <t>Número de Unidades Operacionais e Postos de Atendimentos que prestam atendimento nos departamentos regionais e núcleos regionais.</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>54.63</v>
+        <v>55.58</v>
       </c>
       <c r="G6" t="n">
-        <v>42.08</v>
+        <v>42.81</v>
       </c>
       <c r="H6" t="n">
-        <v>1.71</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>1.58</v>
+        <v>1.61</v>
       </c>
       <c r="J6" t="inlineStr"/>
     </row>
@@ -3677,7 +5485,7 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3687,7 +5495,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Educação Treinamento e Desenvolvimento</t>
+          <t>Comunicação áreas técnicas - Diretoria de Inovação</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -3713,7 +5521,7 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3723,7 +5531,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Gestão e Administração - Gerência de Comunicação Integr</t>
+          <t>Gestão de Pessoal e Encargos - Diretoria de Comunicação</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -3749,7 +5557,7 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -3759,7 +5567,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Gestão de Pessoal e Encargos - Ger de Comunic. Integrad</t>
+          <t>Gestão e Administração - Gerência de Comunicação Integrada, Planej. e Intel</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -3785,7 +5593,7 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3795,7 +5603,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Gestão de Pessoal e Encargos - Ger Comunic. Interna e E</t>
+          <t>Gestão de Pessoal e Encargos - Ger de Comunic. Integrada, Planej. e Inteligência</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -3821,7 +5629,7 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3831,7 +5639,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Gestão e Suporte as Atividades - Ger Comunic. Interna</t>
+          <t>Gestão e Suporte as Atividades - Diretoria de Comunicação</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -3857,17 +5665,17 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Diretoria de Comunicação</t>
+          <t>Diretoria de Inovação</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sistematização e Gestão das Info. - Customer Relationship Management (CRM)</t>
+          <t>Educação Treinamento e Desenvolvimento Diretoria de Inovação</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -3893,35 +5701,35 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Diretoria de Comunicação</t>
+          <t>Diretoria de Inovação</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Gestão de Pessoal e Encargos - Super. de Jornalismo</t>
+          <t>Congresso Internacional de Inovação da Indústria - Convênio CNI/SEBRAE - Entidade</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Número de Unidades Operacionais e Postos de Atendimentos que prestam atendimento nos Departamentos Regionais do SESI e SENAI e Sede das Federações e do IEL</t>
+          <t>Estabelecido em Convênio</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>54.63</v>
+        <v>53.4</v>
       </c>
       <c r="G13" t="n">
-        <v>42.08</v>
+        <v>41.56</v>
       </c>
       <c r="H13" t="n">
-        <v>1.71</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>1.58</v>
+        <v>5.04</v>
       </c>
       <c r="J13" t="inlineStr"/>
     </row>
@@ -3929,35 +5737,35 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Diretoria de Comunicação</t>
+          <t>Diretoria de Inovação</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Gestão e Administração - Super. de Jornalismo</t>
+          <t>Edição 2023 - Prêmio de Inovação - Convênio CNI/SEBRAE - Entidade</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Número de Unidades Operacionais e Postos de Atendimentos que prestam atendimento nos Departamentos Regionais do SESI e SENAI e Sede das Federações e do IEL</t>
+          <t>Estabelecido em Convênio</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>54.63</v>
+        <v>50.55</v>
       </c>
       <c r="G14" t="n">
-        <v>42.08</v>
+        <v>38.71</v>
       </c>
       <c r="H14" t="n">
-        <v>1.71</v>
+        <v>5.7</v>
       </c>
       <c r="I14" t="n">
-        <v>1.58</v>
+        <v>5.04</v>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
@@ -3965,17 +5773,17 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Diretoria de Comunicação</t>
+          <t>Diretoria de Inovação</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Programa de Relacionamento</t>
+          <t>Gestão da Diretoria de Tecnologia e Inovação</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -4001,17 +5809,17 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Diretoria de Comunicação</t>
+          <t>Diretoria de Inovação</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Gestão de Pessoal e Encargos - Ger de Conteúdos Mult</t>
+          <t>Gestão de Pessoal e Encargos - Gerência de Monitoramento e Controle de Projetos</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -4037,35 +5845,35 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Diretoria de Comunicação</t>
+          <t>Diretoria de Inovação</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Gestão de Pessoal e Encargos - Ger de Imprensa</t>
+          <t>Portal e Workshops Mobilização Empresarial pela Inovação (MEI) Tools - Convênio CNI/SEBRAE - Entidade</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Número de Unidades Operacionais e Postos de Atendimentos que prestam atendimento nos Departamentos Regionais do SESI e SENAI e Sede das Federações e do IEL</t>
+          <t>Estabelecido em Convênio</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>54.63</v>
+        <v>50.55</v>
       </c>
       <c r="G17" t="n">
-        <v>42.08</v>
+        <v>38.71</v>
       </c>
       <c r="H17" t="n">
-        <v>1.71</v>
+        <v>5.7</v>
       </c>
       <c r="I17" t="n">
-        <v>1.58</v>
+        <v>5.04</v>
       </c>
       <c r="J17" t="inlineStr"/>
     </row>
@@ -4073,17 +5881,17 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Diretoria de Comunicação</t>
+          <t>Diretoria de Inovação</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Gestão e Administração - Superintendência de Publicidade</t>
+          <t>Gestão de Pessoal e Encargos - Gerência de Mobilização Empresarial</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -4109,17 +5917,17 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Diretoria de Comunicação</t>
+          <t>Diretoria de Inovação</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Gestão de Pessoal e Encargos - Superintendência de Publicidade</t>
+          <t>Gestão de Pessoal e Encargos - Superintendência de Projetos</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -4145,17 +5953,17 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Diretoria de Comunicação</t>
+          <t>Diretoria de Inovação</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Gestão de Pessoal e Encargos - Ger de Criação de Public</t>
+          <t>Gestão da Superintendência de Projetos de Inovação</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -4181,17 +5989,17 @@
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
-          <t>17/02/2025 11:38</t>
+          <t>08/08/2024 16:32</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Diretoria de Comunicação</t>
+          <t>Diretoria de Inovação</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Gestão de Pessoal e Encargos - Ger. de Estratégia de Public</t>
+          <t>Secretaria Executiva da Mobilização Empresarial pela Inovação (MEI)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -4277,7 +6085,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>05/02/2026 16:43</t>
+          <t>27/01/2025 09:44</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4291,10 +6099,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>45124118.82</v>
+        <v>49732898.5</v>
       </c>
       <c r="E2" t="n">
-        <v>46.48</v>
+        <v>52.35</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4307,16 +6115,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>19086188.68</v>
+        <v>30584453.82</v>
       </c>
       <c r="I2" t="n">
-        <v>42.3</v>
+        <v>61.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>05/02/2026 16:43</t>
+          <t>27/01/2025 09:44</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4330,10 +6138,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>45124118.82</v>
+        <v>49732898.5</v>
       </c>
       <c r="E3" t="n">
-        <v>46.48</v>
+        <v>52.35</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4346,16 +6154,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>220809.7</v>
+        <v>610525.66</v>
       </c>
       <c r="I3" t="n">
-        <v>0.49</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>05/02/2026 16:43</t>
+          <t>27/01/2025 09:44</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4369,10 +6177,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>45124118.82</v>
+        <v>49732898.5</v>
       </c>
       <c r="E4" t="n">
-        <v>46.48</v>
+        <v>52.35</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -4394,7 +6202,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>05/02/2026 16:43</t>
+          <t>27/01/2025 09:44</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4408,10 +6216,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>45124118.82</v>
+        <v>49732898.5</v>
       </c>
       <c r="E5" t="n">
-        <v>46.48</v>
+        <v>52.35</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -4433,7 +6241,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05/02/2026 16:43</t>
+          <t>27/01/2025 09:44</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4447,10 +6255,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>45124118.82</v>
+        <v>49732898.5</v>
       </c>
       <c r="E6" t="n">
-        <v>46.48</v>
+        <v>52.35</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -4463,16 +6271,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>7174583.82</v>
+        <v>10473695.89</v>
       </c>
       <c r="I6" t="n">
-        <v>15.9</v>
+        <v>21.06</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05/02/2026 16:43</t>
+          <t>27/01/2025 09:44</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4486,10 +6294,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>45124118.82</v>
+        <v>49732898.5</v>
       </c>
       <c r="E7" t="n">
-        <v>46.48</v>
+        <v>52.35</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -4502,16 +6310,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>5820940.07</v>
+        <v>6284378.66</v>
       </c>
       <c r="I7" t="n">
-        <v>12.9</v>
+        <v>12.64</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05/02/2026 16:43</t>
+          <t>27/01/2025 09:44</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4525,10 +6333,10 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>45124118.82</v>
+        <v>49732898.5</v>
       </c>
       <c r="E8" t="n">
-        <v>46.48</v>
+        <v>52.35</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -4541,16 +6349,16 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>11705301.29</v>
+        <v>1779844.47</v>
       </c>
       <c r="I8" t="n">
-        <v>25.94</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05/02/2026 16:43</t>
+          <t>27/01/2025 09:44</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4564,10 +6372,10 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>45124118.82</v>
+        <v>49732898.5</v>
       </c>
       <c r="E9" t="n">
-        <v>46.48</v>
+        <v>52.35</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -4580,16 +6388,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1116295.26</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>2.47</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05/02/2026 16:43</t>
+          <t>27/01/2025 09:44</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4603,10 +6411,10 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>51961000.5</v>
+        <v>45270715.53</v>
       </c>
       <c r="E10" t="n">
-        <v>53.52</v>
+        <v>47.65</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -4619,16 +6427,16 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>12693866.12</v>
+        <v>11561424.09</v>
       </c>
       <c r="I10" t="n">
-        <v>24.43</v>
+        <v>25.54</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05/02/2026 16:43</t>
+          <t>27/01/2025 09:44</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4642,10 +6450,10 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>51961000.5</v>
+        <v>45270715.53</v>
       </c>
       <c r="E11" t="n">
-        <v>53.52</v>
+        <v>47.65</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -4658,16 +6466,16 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>11570919.17</v>
+        <v>18462203.1</v>
       </c>
       <c r="I11" t="n">
-        <v>22.27</v>
+        <v>40.78</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05/02/2026 16:43</t>
+          <t>27/01/2025 09:44</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4681,10 +6489,10 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>51961000.5</v>
+        <v>45270715.53</v>
       </c>
       <c r="E12" t="n">
-        <v>53.52</v>
+        <v>47.65</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -4697,16 +6505,16 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>27696215.21</v>
+        <v>15247088.34</v>
       </c>
       <c r="I12" t="n">
-        <v>53.3</v>
+        <v>33.68</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05/02/2026 16:43</t>
+          <t>27/01/2025 09:44</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -4720,7 +6528,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>97085119.31999999</v>
+        <v>95003614.03</v>
       </c>
       <c r="E13" t="n">
         <v>100</v>
@@ -4814,7 +6622,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4834,7 +6642,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -4865,7 +6673,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4885,7 +6693,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -4916,7 +6724,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4936,7 +6744,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -4954,20 +6762,20 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>10556450.04</v>
+        <v>35371852.53</v>
       </c>
       <c r="K4" t="n">
-        <v>15224664</v>
+        <v>28106750.57</v>
       </c>
       <c r="L4" t="n">
-        <v>144.2</v>
+        <v>79.5</v>
       </c>
       <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4987,7 +6795,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -5018,7 +6826,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -5038,7 +6846,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -5069,7 +6877,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -5089,7 +6897,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -5120,7 +6928,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>22/01/2026 11:34</t>
+          <t>27/01/2025 09:55</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -5140,7 +6948,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2025</t>
+          <t>Valores Aprovados no Plano de Ação e Orçamento Suplementado 2024</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -5158,15 +6966,258 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>10556450.04</v>
+        <v>35371852.53</v>
       </c>
       <c r="K8" t="n">
-        <v>15224664</v>
+        <v>28106750.57</v>
       </c>
       <c r="L8" t="n">
-        <v>144.2</v>
+        <v>79.5</v>
       </c>
       <c r="M8" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>codigoVwRelacaoDirigenteEmpregado</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sgEntidadeNacional</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>cargo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>sgEntidadeRegional</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>dataPublicacao</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>sgModulo</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>nomeModulo</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>titulo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>nota</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>fonte</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>analise</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>extra</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>entidadeRegional.id</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>entidadeRegional.siglaRegional</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>entidadeRegional.codigoNacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1102</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ANTÔNIO RICARDO ALVAREZ ALBAN¹</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Presidente do Conselho Nacional</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>RL_DRG_GEST</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>RELAÇÃO DE DIRIGENTES - GESTÃO</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Relação de Dirigentes - Gestão</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>1. Não recebe remuneração.</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Superintendência de Desenvolvimento Humano</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="n">
+        <v>3</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1103</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SENAI</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GUSTAVO LEAL SALES FILHO</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Diretor Geral do SENAI-DN</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>01/01/2024 11:00:00</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>RL_DRG_GEST</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>RELAÇÃO DE DIRIGENTES - GESTÃO</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Relação de Dirigentes - Gestão</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>1. Não recebe remuneração.</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Superintendência de Desenvolvimento Humano</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="n">
+        <v>3</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SENAI-DN</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>